<commit_message>
Fix FY2023 cost-of-sales citation to reference reclassified 10-K filing
</commit_message>
<xml_diff>
--- a/model/WC_Benchmark_Dashboard.xlsx
+++ b/model/WC_Benchmark_Dashboard.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbcc2df38bfc14c50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ratios" sheetId="2" r:id="R8299a424926e4cae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Financials" sheetId="3" r:id="R1c48ac5abe5846f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="4" r:id="R953854436bb5495b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R78827611df3c4040"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ratios" sheetId="2" r:id="R0551f2aa08884238"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Financials" sheetId="3" r:id="R09c46f81fa904e8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="4" r:id="R034e8dd809ce4bb2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1554,13 +1554,13 @@
         <x:v>2024-02-03</x:v>
       </x:c>
       <x:c r="H3" t="str">
-        <x:v>2024-03-13</x:v>
+        <x:v>2025-03-12</x:v>
       </x:c>
       <x:c r="I3" t="str">
-        <x:v>0000027419-24-000032</x:v>
+        <x:v>0000027419-25-000018</x:v>
       </x:c>
       <x:c r="J3" t="str">
-        <x:v>https://www.sec.gov/Archives/edgar/data/27419/000002741924000032/tgt-20240203.htm</x:v>
+        <x:v>https://www.sec.gov/Archives/edgar/data/27419/000002741925000018/tgt-20250201.htm</x:v>
       </x:c>
       <x:c r="K3" s="4" t="n">
         <x:v>107412</x:v>
@@ -1578,7 +1578,7 @@
         <x:v>12098</x:v>
       </x:c>
       <x:c r="P3" t="str">
-        <x:v>No separate trade AR line; treated as immaterial/absent for DSO</x:v>
+        <x:v>FY2023 cost of sales uses the $92m reclassified presentation reported in Target's FY2024 Form 10-K; no separate trade AR line</x:v>
       </x:c>
       <x:c r="Q3" t="str">
         <x:v>RevenueFromContractWithCustomerExcludingAssessedTax</x:v>
@@ -2768,7 +2768,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R927d134118254eae"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re23860fc048e4b05"/>
 </x:worksheet>
 </file>
 

</xml_diff>